<commit_message>
Daily EOD data and reports for 2026-08-10
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260810.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260810.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.56</v>
+        <v>1.555</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>1.30%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>238962.36</v>
+        <v>238196.45</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>3829.53</v>
+        <v>3063.62</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.48%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>165900</v>
+        <v>165200</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-3500</v>
+        <v>-4200</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.18</v>
+        <v>1.195</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.31%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>67800.44</v>
+        <v>68662.31</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4022.06</v>
+        <v>4883.93</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>63.52</v>
+        <v>63.83</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.55</v>
+        <v>0.86</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.87%</t>
+          <t>1.37%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>702848.8</v>
+        <v>706278.95</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>6085.75</v>
+        <v>9515.9</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>175.39</v>
+        <v>176.61</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.62</v>
+        <v>-1.4</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.47%</t>
+          <t>-0.79%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.905</v>
+        <v>0.9</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.035</v>
+        <v>0.03</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9050</v>
+        <v>9000</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>36.64</v>
+        <v>36.565</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-1.29</v>
+        <v>-1.365</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-3.40%</t>
+          <t>-3.60%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.95</v>
+        <v>31.94</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.19%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41151.6</v>
+        <v>41138.72</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>90.16</v>
+        <v>77.28</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1763741.47</v>
+        <v>1766504.7</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>11547.59</v>
+        <v>14310.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>